<commit_message>
add the check the end in import excel file for all invoices
</commit_message>
<xml_diff>
--- a/hddt-SES/src/main/resources/static/cttncn/MauUploadCT_TNCN-TT78.xlsx
+++ b/hddt-SES/src/main/resources/static/cttncn/MauUploadCT_TNCN-TT78.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11730"/>
+    <workbookView windowWidth="28800" windowHeight="12180"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -293,7 +293,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="39">
   <si>
     <t>MaCT(*)</t>
   </si>
@@ -398,6 +398,9 @@
   </si>
   <si>
     <t>Địa chỉ B</t>
+  </si>
+  <si>
+    <t>END</t>
   </si>
   <si>
     <t>Cá nhân cư trú</t>
@@ -419,7 +422,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -429,13 +432,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -585,6 +581,17 @@
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
     <font>
       <b/>
@@ -592,19 +599,8 @@
       <name val="Tahoma"/>
       <charset val="134"/>
     </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
   </fonts>
-  <fills count="36">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -691,19 +687,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -925,95 +909,101 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1022,10 +1012,10 @@
     <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1034,10 +1024,10 @@
     <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1046,10 +1036,10 @@
     <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1058,13 +1048,7 @@
     <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1410,8 +1394,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:R3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="2"/>
+  <dimension ref="A1:R4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="3"/>
   <cols>
     <col min="2" max="2" width="14.7238095238095" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
@@ -1592,6 +1576,11 @@
         <v>20000000</v>
       </c>
     </row>
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="portrait"/>
@@ -1612,18 +1601,18 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat:   - add select option mstncn when import excel file on cttncn   - update excel file  on cttncn   - update handle import and load excelfile
</commit_message>
<xml_diff>
--- a/hddt-SES/src/main/resources/static/cttncn/MauUploadCT_TNCN-TT78.xlsx
+++ b/hddt-SES/src/main/resources/static/cttncn/MauUploadCT_TNCN-TT78.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180"/>
+    <workbookView windowWidth="23040" windowHeight="8940"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,6 +31,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>VAN HAU</author>
+    <author>trann</author>
     <author>ASIA</author>
   </authors>
   <commentList>
@@ -117,7 +118,33 @@
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0">
+    <comment ref="F1" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="11"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>Số điện thoại liên hệ</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="11"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>Email liên hệ</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -130,7 +157,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0">
+    <comment ref="I1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -143,7 +170,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0">
+    <comment ref="J1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -156,7 +183,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0">
+    <comment ref="K1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -169,7 +196,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J1" authorId="1">
+    <comment ref="L1" authorId="2">
       <text>
         <r>
           <rPr>
@@ -184,7 +211,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K1" authorId="0">
+    <comment ref="M1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -197,7 +224,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0">
+    <comment ref="N1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -206,11 +233,11 @@
             <rFont val="Tahoma"/>
             <charset val="1"/>
           </rPr>
-          <t>Từ ngày</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M1" authorId="1">
+          <t>Từ ngày (dd/mm/yyyy)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="2">
       <text>
         <r>
           <rPr>
@@ -219,11 +246,11 @@
             <rFont val="Tahoma"/>
             <charset val="134"/>
           </rPr>
-          <t>Đến ngày</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N1" authorId="1">
+          <t>Đến ngày (dd/mm/yyyy)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="2">
       <text>
         <r>
           <rPr>
@@ -236,7 +263,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O1" authorId="0">
+    <comment ref="Q1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -249,7 +276,20 @@
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="0">
+    <comment ref="R1" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="11"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>Khoản đóng từ thiện, nhân đạo, khuyến học</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -262,7 +302,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0">
+    <comment ref="T1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -275,7 +315,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R1" authorId="1">
+    <comment ref="U1" authorId="2">
       <text>
         <r>
           <rPr>
@@ -293,7 +333,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="44">
   <si>
     <t>MaCT(*)</t>
   </si>
@@ -310,6 +350,12 @@
     <t>DiaChiNV</t>
   </si>
   <si>
+    <t>SDTLienHe</t>
+  </si>
+  <si>
+    <t>EmailLienHe</t>
+  </si>
+  <si>
     <t>CMND-CCCD(*)</t>
   </si>
   <si>
@@ -340,6 +386,9 @@
     <t>KhoanDongBHBB</t>
   </si>
   <si>
+    <t>KhoanDongTThienNDaoKHoc</t>
+  </si>
+  <si>
     <t>TongTNChiuThuePhaiKT(*)</t>
   </si>
   <si>
@@ -362,6 +411,12 @@
   </si>
   <si>
     <t>Địa chỉ A</t>
+  </si>
+  <si>
+    <t>0911122233</t>
+  </si>
+  <si>
+    <t>example@gmail.com</t>
   </si>
   <si>
     <t>xxxxxxxxx</t>
@@ -422,7 +477,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -589,15 +644,21 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="9"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
     </font>
   </fonts>
   <fills count="34">
@@ -1052,13 +1113,13 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1067,6 +1128,7 @@
     <xf numFmtId="1" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6"/>
     <xf numFmtId="1" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1074,6 +1136,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="49">
@@ -1394,27 +1457,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:U4"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="3"/>
   <cols>
     <col min="2" max="2" width="14.7238095238095" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="12.7238095238095" customWidth="1"/>
-    <col min="5" max="6" width="19.1809523809524" customWidth="1"/>
-    <col min="7" max="7" width="15.2666666666667" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="12.8190476190476" customWidth="1"/>
-    <col min="10" max="10" width="22.1809523809524" style="2" customWidth="1"/>
-    <col min="11" max="11" width="15.4571428571429" customWidth="1"/>
-    <col min="12" max="13" width="14" style="3" customWidth="1"/>
-    <col min="14" max="14" width="20.1809523809524" customWidth="1"/>
-    <col min="15" max="15" width="20.8190476190476" customWidth="1"/>
-    <col min="16" max="16" width="23.2666666666667" style="4" customWidth="1"/>
-    <col min="17" max="17" width="24.5428571428571" style="5" customWidth="1"/>
-    <col min="18" max="18" width="19.8190476190476" customWidth="1"/>
+    <col min="5" max="5" width="19.1809523809524" customWidth="1"/>
+    <col min="6" max="6" width="19.1809523809524" style="2" customWidth="1"/>
+    <col min="7" max="7" width="21.5714285714286" style="2" customWidth="1"/>
+    <col min="8" max="8" width="19.1809523809524" customWidth="1"/>
+    <col min="9" max="9" width="15.2666666666667" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="12.8190476190476" customWidth="1"/>
+    <col min="12" max="12" width="22.1809523809524" style="3" customWidth="1"/>
+    <col min="13" max="13" width="15.4571428571429" customWidth="1"/>
+    <col min="14" max="15" width="14" style="2" customWidth="1"/>
+    <col min="16" max="16" width="20.1809523809524" customWidth="1"/>
+    <col min="17" max="17" width="20.8190476190476" customWidth="1"/>
+    <col min="18" max="18" width="29.1428571428571" customWidth="1"/>
+    <col min="19" max="19" width="23.2666666666667" style="4" customWidth="1"/>
+    <col min="20" max="20" width="24.5428571428571" style="5" customWidth="1"/>
+    <col min="21" max="21" width="19.8190476190476" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:21">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1430,10 +1497,10 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="7" t="s">
@@ -1445,143 +1512,167 @@
       <c r="J1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="K1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="P1" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="9" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="9" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
+      <c r="S1" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="10" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="2" spans="1:18">
+    <row r="2" spans="1:21">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G2" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>27</v>
       </c>
       <c r="H2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I2" t="s">
+        <v>29</v>
+      </c>
+      <c r="J2" t="s">
+        <v>30</v>
+      </c>
+      <c r="K2" t="s">
+        <v>31</v>
+      </c>
+      <c r="L2" s="3">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>2023</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="S2" s="11">
+        <v>20000000</v>
+      </c>
+      <c r="T2" s="11">
+        <v>20000000</v>
+      </c>
+      <c r="U2" s="11">
+        <v>20000000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21">
+      <c r="A3" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="J2" s="2">
-        <v>1</v>
-      </c>
-      <c r="K2">
+      <c r="G3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" t="s">
+        <v>30</v>
+      </c>
+      <c r="K3" t="s">
+        <v>31</v>
+      </c>
+      <c r="L3" s="3">
+        <v>2</v>
+      </c>
+      <c r="M3">
         <v>2023</v>
       </c>
-      <c r="L2" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="N2" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="P2" s="10">
+      <c r="N3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="S3" s="11">
         <v>20000000</v>
       </c>
-      <c r="Q2" s="10">
+      <c r="T3" s="11">
         <v>20000000</v>
       </c>
-      <c r="R2" s="10">
-        <v>20000000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18">
-      <c r="A3" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G3" t="s">
-        <v>24</v>
-      </c>
-      <c r="H3" t="s">
-        <v>25</v>
-      </c>
-      <c r="I3" t="s">
-        <v>26</v>
-      </c>
-      <c r="J3" s="2">
-        <v>2</v>
-      </c>
-      <c r="K3">
-        <v>2023</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="P3" s="10">
-        <v>20000000</v>
-      </c>
-      <c r="Q3" s="10">
-        <v>20000000</v>
-      </c>
-      <c r="R3" s="10">
+      <c r="U3" s="11">
         <v>20000000</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G2" r:id="rId3" display="example@gmail.com"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="portrait"/>
   <headerFooter/>
@@ -1601,18 +1692,18 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: - update ui on cttncn crud - update sendmail on cttncn - update handle add and search employee on cttncn crud - update excel file when import on cttncn - updata load data from excel file when import on cttncn - update label on mahd crud
</commit_message>
<xml_diff>
--- a/hddt-SES/src/main/resources/static/cttncn/MauUploadCT_TNCN-TT78.xlsx
+++ b/hddt-SES/src/main/resources/static/cttncn/MauUploadCT_TNCN-TT78.xlsx
@@ -144,7 +144,20 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0">
+    <comment ref="H1" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="11"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>Cách nhau bởi dấu ,</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -157,7 +170,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0">
+    <comment ref="J1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -170,7 +183,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J1" authorId="0">
+    <comment ref="K1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -183,7 +196,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K1" authorId="0">
+    <comment ref="L1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -196,7 +209,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="2">
+    <comment ref="M1" authorId="2">
       <text>
         <r>
           <rPr>
@@ -211,7 +224,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0">
+    <comment ref="N1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -224,7 +237,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0">
+    <comment ref="O1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -237,7 +250,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O1" authorId="2">
+    <comment ref="P1" authorId="2">
       <text>
         <r>
           <rPr>
@@ -250,7 +263,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="2">
+    <comment ref="Q1" authorId="2">
       <text>
         <r>
           <rPr>
@@ -263,7 +276,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0">
+    <comment ref="R1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -276,7 +289,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R1" authorId="1">
+    <comment ref="S1" authorId="1">
       <text>
         <r>
           <rPr>
@@ -289,7 +302,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S1" authorId="0">
+    <comment ref="T1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -302,7 +315,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T1" authorId="0">
+    <comment ref="U1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -315,7 +328,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="U1" authorId="2">
+    <comment ref="V1" authorId="2">
       <text>
         <r>
           <rPr>
@@ -333,7 +346,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="45">
   <si>
     <t>MaCT(*)</t>
   </si>
@@ -354,6 +367,9 @@
   </si>
   <si>
     <t>EmailLienHe</t>
+  </si>
+  <si>
+    <t>EmailCC</t>
   </si>
   <si>
     <t>CMND-CCCD(*)</t>
@@ -638,6 +654,11 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="9"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
@@ -645,20 +666,15 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Times New Roman"/>
-      <charset val="0"/>
     </font>
   </fonts>
   <fills count="34">
@@ -1128,7 +1144,7 @@
     <xf numFmtId="1" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyAlignment="1"/>
     <xf numFmtId="1" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1457,7 +1473,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:V4"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="3"/>
   <cols>
     <col min="2" max="2" width="14.7238095238095" customWidth="1"/>
@@ -1465,23 +1481,23 @@
     <col min="4" max="4" width="12.7238095238095" customWidth="1"/>
     <col min="5" max="5" width="19.1809523809524" customWidth="1"/>
     <col min="6" max="6" width="19.1809523809524" style="2" customWidth="1"/>
-    <col min="7" max="7" width="21.5714285714286" style="2" customWidth="1"/>
-    <col min="8" max="8" width="19.1809523809524" customWidth="1"/>
-    <col min="9" max="9" width="15.2666666666667" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="12.8190476190476" customWidth="1"/>
-    <col min="12" max="12" width="22.1809523809524" style="3" customWidth="1"/>
-    <col min="13" max="13" width="15.4571428571429" customWidth="1"/>
-    <col min="14" max="15" width="14" style="2" customWidth="1"/>
-    <col min="16" max="16" width="20.1809523809524" customWidth="1"/>
-    <col min="17" max="17" width="20.8190476190476" customWidth="1"/>
-    <col min="18" max="18" width="29.1428571428571" customWidth="1"/>
-    <col min="19" max="19" width="23.2666666666667" style="4" customWidth="1"/>
-    <col min="20" max="20" width="24.5428571428571" style="5" customWidth="1"/>
-    <col min="21" max="21" width="19.8190476190476" customWidth="1"/>
+    <col min="7" max="8" width="21.5714285714286" style="2" customWidth="1"/>
+    <col min="9" max="9" width="19.1809523809524" customWidth="1"/>
+    <col min="10" max="10" width="15.2666666666667" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="12.8190476190476" customWidth="1"/>
+    <col min="13" max="13" width="22.1809523809524" style="3" customWidth="1"/>
+    <col min="14" max="14" width="15.4571428571429" customWidth="1"/>
+    <col min="15" max="16" width="14" style="2" customWidth="1"/>
+    <col min="17" max="17" width="20.1809523809524" customWidth="1"/>
+    <col min="18" max="18" width="20.8190476190476" customWidth="1"/>
+    <col min="19" max="19" width="29.1428571428571" customWidth="1"/>
+    <col min="20" max="20" width="23.2666666666667" style="4" customWidth="1"/>
+    <col min="21" max="21" width="24.5428571428571" style="5" customWidth="1"/>
+    <col min="22" max="22" width="19.8190476190476" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21">
+    <row r="1" spans="1:22">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1503,7 +1519,7 @@
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="7" t="s">
@@ -1518,25 +1534,25 @@
       <c r="L1" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="M1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="9" t="s">
         <v>13</v>
       </c>
       <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="10" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="10" t="s">
         <v>16</v>
       </c>
       <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="10" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
       <c r="T1" s="10" t="s">
@@ -1545,32 +1561,33 @@
       <c r="U1" s="10" t="s">
         <v>20</v>
       </c>
+      <c r="V1" s="10" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="2" spans="1:21">
+    <row r="2" spans="1:22">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="H2" t="s">
         <v>28</v>
       </c>
+      <c r="H2" s="8"/>
       <c r="I2" t="s">
         <v>29</v>
       </c>
@@ -1580,23 +1597,23 @@
       <c r="K2" t="s">
         <v>31</v>
       </c>
-      <c r="L2" s="3">
+      <c r="L2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M2" s="3">
         <v>1</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>2023</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="O2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="P2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="S2" s="11">
-        <v>20000000</v>
+      <c r="Q2" s="5" t="s">
+        <v>35</v>
       </c>
       <c r="T2" s="11">
         <v>20000000</v>
@@ -1604,32 +1621,33 @@
       <c r="U2" s="11">
         <v>20000000</v>
       </c>
+      <c r="V2" s="11">
+        <v>20000000</v>
+      </c>
     </row>
-    <row r="3" spans="1:21">
+    <row r="3" spans="1:22">
       <c r="A3" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G3" t="s">
-        <v>27</v>
-      </c>
-      <c r="H3" t="s">
         <v>28</v>
       </c>
+      <c r="H3"/>
       <c r="I3" t="s">
         <v>29</v>
       </c>
@@ -1639,34 +1657,37 @@
       <c r="K3" t="s">
         <v>31</v>
       </c>
-      <c r="L3" s="3">
+      <c r="L3" t="s">
+        <v>32</v>
+      </c>
+      <c r="M3" s="3">
         <v>2</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>2023</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="O3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="P3" s="5" t="s">
+      <c r="P3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="S3" s="11">
-        <v>20000000</v>
+      <c r="Q3" s="5" t="s">
+        <v>35</v>
       </c>
       <c r="T3" s="11">
         <v>20000000</v>
       </c>
       <c r="U3" s="11">
+        <v>20000000</v>
+      </c>
+      <c r="V3" s="11">
         <v>20000000</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1692,18 +1713,18 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>